<commit_message>
Template and Tech requirement updates
</commit_message>
<xml_diff>
--- a/Analysis Examples/Cardex-Variance-Item-Analysis.xlsx
+++ b/Analysis Examples/Cardex-Variance-Item-Analysis.xlsx
@@ -1531,7 +1531,7 @@
     <row r="2" ht="38" customHeight="1" s="65">
       <c r="A2" s="126" t="inlineStr">
         <is>
-          <t>Item 555 — Branch IDM, Location MLD</t>
+          <t>Item 99955 — Branch BR1, Location LOC1</t>
         </is>
       </c>
     </row>
@@ -1545,7 +1545,7 @@
     <row r="4" ht="18" customHeight="1" s="65">
       <c r="A4" s="128" t="inlineStr">
         <is>
-          <t>GL Class  COLC          GL Account  1000000.141000.CC          Std Cost  $5.72/LB</t>
+          <t>GL Class  COLC          GL Account  9100000.611000.A1          Std Cost  $5.72/LB</t>
         </is>
       </c>
     </row>
@@ -1586,7 +1586,7 @@
     <row r="10" ht="130" customHeight="1" s="65">
       <c r="A10" s="134" t="inlineStr">
         <is>
-          <t>The F4111 item ledger for Item 555 shows a current running balance of 10.35 LB worth $59.21 — but RapidReconciler reports the F41021 on-hand table is 10.35 LB short.
+          <t>The F4111 item ledger for Item 99955 shows a current running balance of 10.35 LB worth $59.21 — but RapidReconciler reports the F41021 on-hand table is 10.35 LB short.
 The entire current ledger balance is the variance: F41021 is effectively at 0 LB while F4111 says 10.35 LB.  Standard cost has held steady at $5.72/LB throughout, so the dollar gap is essentially the quantity gap × standard cost.  Fixing the quantity will clear most of the dollar variance, with a small residual to clean up.</t>
         </is>
       </c>
@@ -1625,11 +1625,11 @@
     <row r="14" ht="240" customHeight="1" s="65">
       <c r="A14" s="134" t="inlineStr">
         <is>
-          <t>Step 1.  Confirm F41021 on-hand qty for Item 555 / Branch IDM / Location MLD really is 0 LB.  If it isn’t, run a cycle count or adjust the quantity manually, then re-evaluate after the next RapidReconciler refresh cycle.
+          <t>Step 1.  Confirm F41021 on-hand qty for Item 99955 / Branch BR1 / Location LOC1 really is 0 LB.  If it isn’t, run a cycle count or adjust the quantity manually, then re-evaluate after the next RapidReconciler refresh cycle.
 Step 2.  View the item on the item ledger screen in JD Edwards, display all rows, and export to Excel.  Then perform an analysis using the “Handling Cardex Variance Guide” to obtain the current quantity and amount variances — these are the figures to use for the corrections in the steps below, since the variance shown here may have moved since this analysis was generated.
 Step 3.  Request an F41021 SQL correction from IT using the current quantity variance from Step 2 (DBA support required — confirm F4111 is the accurate record before proceeding).
 Step 4.  If there are any residual amounts after the quantity correction, perform a dollars-only adjustment to clear.
-Step 5.  After the corrections, run Re-Roll on the RapidReconciler As Of page for all locations for Item 555 and confirm QtyVar and AmtVar both go to zero on the next refresh.</t>
+Step 5.  After the corrections, run Re-Roll on the RapidReconciler As Of page for all locations for Item 99955 and confirm QtyVar and AmtVar both go to zero on the next refresh.</t>
         </is>
       </c>
       <c r="B14" s="135" t="n"/>
@@ -1870,7 +1870,7 @@
     <row r="1" ht="27.95" customHeight="1" s="65">
       <c r="A1" s="67" t="inlineStr">
         <is>
-          <t>Item Roll Forward — Item 555 / Branch IDM / Location MLD  |  Cost Method 07 (Standard)  |  Cost Level 2</t>
+          <t>Item Roll Forward — Item 99955 / Branch BR1 / Location LOC1  |  Cost Method 07 (Standard)  |  Cost Level 2</t>
         </is>
       </c>
     </row>
@@ -1989,7 +1989,7 @@
       </c>
       <c r="B3" s="151" t="inlineStr">
         <is>
-          <t>1000000.141000.CC</t>
+          <t>9100000.611000.A1</t>
         </is>
       </c>
       <c r="C3" s="152" t="n">
@@ -1997,17 +1997,17 @@
       </c>
       <c r="D3" s="151" t="inlineStr">
         <is>
-          <t>IDM</t>
+          <t>BR1</t>
         </is>
       </c>
       <c r="E3" s="151" t="inlineStr">
         <is>
-          <t>555</t>
+          <t>99955</t>
         </is>
       </c>
       <c r="F3" s="151" t="inlineStr">
         <is>
-          <t>MLD</t>
+          <t>LOC1</t>
         </is>
       </c>
       <c r="G3" s="151" t="n"/>
@@ -2068,7 +2068,7 @@
       </c>
       <c r="B4" s="158" t="inlineStr">
         <is>
-          <t>1000000.141000.CC</t>
+          <t>9100000.611000.A1</t>
         </is>
       </c>
       <c r="C4" s="159" t="n">
@@ -2076,17 +2076,17 @@
       </c>
       <c r="D4" s="158" t="inlineStr">
         <is>
-          <t>IDM</t>
+          <t>BR1</t>
         </is>
       </c>
       <c r="E4" s="158" t="inlineStr">
         <is>
-          <t>555</t>
+          <t>99955</t>
         </is>
       </c>
       <c r="F4" s="158" t="inlineStr">
         <is>
-          <t>MLD</t>
+          <t>LOC1</t>
         </is>
       </c>
       <c r="G4" s="158" t="n"/>
@@ -2107,7 +2107,7 @@
       </c>
       <c r="K4" s="158" t="inlineStr">
         <is>
-          <t>WHS A MLD</t>
+          <t>WHS A LOC1</t>
         </is>
       </c>
       <c r="L4" s="161" t="n">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="B5" s="158" t="inlineStr">
         <is>
-          <t>1000000.141000.CC</t>
+          <t>9100000.611000.A1</t>
         </is>
       </c>
       <c r="C5" s="159" t="n">
@@ -2157,17 +2157,17 @@
       </c>
       <c r="D5" s="158" t="inlineStr">
         <is>
-          <t>IDM</t>
+          <t>BR1</t>
         </is>
       </c>
       <c r="E5" s="158" t="inlineStr">
         <is>
-          <t>555</t>
+          <t>99955</t>
         </is>
       </c>
       <c r="F5" s="158" t="inlineStr">
         <is>
-          <t>MLD</t>
+          <t>LOC1</t>
         </is>
       </c>
       <c r="G5" s="158" t="n"/>
@@ -2230,7 +2230,7 @@
       </c>
       <c r="B6" s="158" t="inlineStr">
         <is>
-          <t>1000000.141000.CC</t>
+          <t>9100000.611000.A1</t>
         </is>
       </c>
       <c r="C6" s="159" t="n">
@@ -2238,17 +2238,17 @@
       </c>
       <c r="D6" s="158" t="inlineStr">
         <is>
-          <t>IDM</t>
+          <t>BR1</t>
         </is>
       </c>
       <c r="E6" s="158" t="inlineStr">
         <is>
-          <t>555</t>
+          <t>99955</t>
         </is>
       </c>
       <c r="F6" s="158" t="inlineStr">
         <is>
-          <t>MLD</t>
+          <t>LOC1</t>
         </is>
       </c>
       <c r="G6" s="158" t="n"/>
@@ -2311,7 +2311,7 @@
       </c>
       <c r="B7" s="158" t="inlineStr">
         <is>
-          <t>1000000.141000.CC</t>
+          <t>9100000.611000.A1</t>
         </is>
       </c>
       <c r="C7" s="159" t="n">
@@ -2319,17 +2319,17 @@
       </c>
       <c r="D7" s="158" t="inlineStr">
         <is>
-          <t>IDM</t>
+          <t>BR1</t>
         </is>
       </c>
       <c r="E7" s="158" t="inlineStr">
         <is>
-          <t>555</t>
+          <t>99955</t>
         </is>
       </c>
       <c r="F7" s="158" t="inlineStr">
         <is>
-          <t>MLD</t>
+          <t>LOC1</t>
         </is>
       </c>
       <c r="G7" s="158" t="n"/>
@@ -2392,7 +2392,7 @@
       </c>
       <c r="B8" s="158" t="inlineStr">
         <is>
-          <t>1000000.141000.CC</t>
+          <t>9100000.611000.A1</t>
         </is>
       </c>
       <c r="C8" s="159" t="n">
@@ -2400,17 +2400,17 @@
       </c>
       <c r="D8" s="158" t="inlineStr">
         <is>
-          <t>IDM</t>
+          <t>BR1</t>
         </is>
       </c>
       <c r="E8" s="158" t="inlineStr">
         <is>
-          <t>555</t>
+          <t>99955</t>
         </is>
       </c>
       <c r="F8" s="158" t="inlineStr">
         <is>
-          <t>MLD</t>
+          <t>LOC1</t>
         </is>
       </c>
       <c r="G8" s="158" t="n"/>
@@ -2473,7 +2473,7 @@
       </c>
       <c r="B9" s="158" t="inlineStr">
         <is>
-          <t>1000000.141000.CC</t>
+          <t>9100000.611000.A1</t>
         </is>
       </c>
       <c r="C9" s="159" t="n">
@@ -2481,17 +2481,17 @@
       </c>
       <c r="D9" s="158" t="inlineStr">
         <is>
-          <t>IDM</t>
+          <t>BR1</t>
         </is>
       </c>
       <c r="E9" s="158" t="inlineStr">
         <is>
-          <t>555</t>
+          <t>99955</t>
         </is>
       </c>
       <c r="F9" s="158" t="inlineStr">
         <is>
-          <t>MLD</t>
+          <t>LOC1</t>
         </is>
       </c>
       <c r="G9" s="158" t="n"/>
@@ -2554,7 +2554,7 @@
       </c>
       <c r="B10" s="158" t="inlineStr">
         <is>
-          <t>1000000.141000.CC</t>
+          <t>9100000.611000.A1</t>
         </is>
       </c>
       <c r="C10" s="159" t="n">
@@ -2562,17 +2562,17 @@
       </c>
       <c r="D10" s="158" t="inlineStr">
         <is>
-          <t>IDM</t>
+          <t>BR1</t>
         </is>
       </c>
       <c r="E10" s="158" t="inlineStr">
         <is>
-          <t>555</t>
+          <t>99955</t>
         </is>
       </c>
       <c r="F10" s="158" t="inlineStr">
         <is>
-          <t>MLD</t>
+          <t>LOC1</t>
         </is>
       </c>
       <c r="G10" s="158" t="n"/>
@@ -2635,7 +2635,7 @@
       </c>
       <c r="B11" s="158" t="inlineStr">
         <is>
-          <t>1000000.141000.CC</t>
+          <t>9100000.611000.A1</t>
         </is>
       </c>
       <c r="C11" s="159" t="n">
@@ -2643,17 +2643,17 @@
       </c>
       <c r="D11" s="158" t="inlineStr">
         <is>
-          <t>IDM</t>
+          <t>BR1</t>
         </is>
       </c>
       <c r="E11" s="158" t="inlineStr">
         <is>
-          <t>555</t>
+          <t>99955</t>
         </is>
       </c>
       <c r="F11" s="158" t="inlineStr">
         <is>
-          <t>MLD</t>
+          <t>LOC1</t>
         </is>
       </c>
       <c r="G11" s="158" t="n"/>
@@ -2716,7 +2716,7 @@
       </c>
       <c r="B12" s="158" t="inlineStr">
         <is>
-          <t>1000000.141000.CC</t>
+          <t>9100000.611000.A1</t>
         </is>
       </c>
       <c r="C12" s="159" t="n">
@@ -2724,17 +2724,17 @@
       </c>
       <c r="D12" s="158" t="inlineStr">
         <is>
-          <t>IDM</t>
+          <t>BR1</t>
         </is>
       </c>
       <c r="E12" s="158" t="inlineStr">
         <is>
-          <t>555</t>
+          <t>99955</t>
         </is>
       </c>
       <c r="F12" s="158" t="inlineStr">
         <is>
-          <t>MLD</t>
+          <t>LOC1</t>
         </is>
       </c>
       <c r="G12" s="158" t="n"/>
@@ -2797,7 +2797,7 @@
       </c>
       <c r="B13" s="158" t="inlineStr">
         <is>
-          <t>1000000.141000.CC</t>
+          <t>9100000.611000.A1</t>
         </is>
       </c>
       <c r="C13" s="159" t="n">
@@ -2805,17 +2805,17 @@
       </c>
       <c r="D13" s="158" t="inlineStr">
         <is>
-          <t>IDM</t>
+          <t>BR1</t>
         </is>
       </c>
       <c r="E13" s="158" t="inlineStr">
         <is>
-          <t>555</t>
+          <t>99955</t>
         </is>
       </c>
       <c r="F13" s="158" t="inlineStr">
         <is>
-          <t>MLD</t>
+          <t>LOC1</t>
         </is>
       </c>
       <c r="G13" s="158" t="n"/>
@@ -2878,7 +2878,7 @@
       </c>
       <c r="B14" s="158" t="inlineStr">
         <is>
-          <t>1000000.141000.CC</t>
+          <t>9100000.611000.A1</t>
         </is>
       </c>
       <c r="C14" s="159" t="n">
@@ -2886,17 +2886,17 @@
       </c>
       <c r="D14" s="158" t="inlineStr">
         <is>
-          <t>IDM</t>
+          <t>BR1</t>
         </is>
       </c>
       <c r="E14" s="158" t="inlineStr">
         <is>
-          <t>555</t>
+          <t>99955</t>
         </is>
       </c>
       <c r="F14" s="158" t="inlineStr">
         <is>
-          <t>MLD</t>
+          <t>LOC1</t>
         </is>
       </c>
       <c r="G14" s="158" t="n"/>
@@ -2959,7 +2959,7 @@
       </c>
       <c r="B15" s="158" t="inlineStr">
         <is>
-          <t>1000000.141000.CC</t>
+          <t>9100000.611000.A1</t>
         </is>
       </c>
       <c r="C15" s="159" t="n">
@@ -2967,17 +2967,17 @@
       </c>
       <c r="D15" s="158" t="inlineStr">
         <is>
-          <t>IDM</t>
+          <t>BR1</t>
         </is>
       </c>
       <c r="E15" s="158" t="inlineStr">
         <is>
-          <t>555</t>
+          <t>99955</t>
         </is>
       </c>
       <c r="F15" s="158" t="inlineStr">
         <is>
-          <t>MLD</t>
+          <t>LOC1</t>
         </is>
       </c>
       <c r="G15" s="158" t="n"/>
@@ -3040,7 +3040,7 @@
       </c>
       <c r="B16" s="158" t="inlineStr">
         <is>
-          <t>1000000.141000.CC</t>
+          <t>9100000.611000.A1</t>
         </is>
       </c>
       <c r="C16" s="159" t="n">
@@ -3048,17 +3048,17 @@
       </c>
       <c r="D16" s="158" t="inlineStr">
         <is>
-          <t>IDM</t>
+          <t>BR1</t>
         </is>
       </c>
       <c r="E16" s="158" t="inlineStr">
         <is>
-          <t>555</t>
+          <t>99955</t>
         </is>
       </c>
       <c r="F16" s="158" t="inlineStr">
         <is>
-          <t>MLD</t>
+          <t>LOC1</t>
         </is>
       </c>
       <c r="G16" s="158" t="n"/>
@@ -3121,7 +3121,7 @@
       </c>
       <c r="B17" s="158" t="inlineStr">
         <is>
-          <t>1000000.141000.CC</t>
+          <t>9100000.611000.A1</t>
         </is>
       </c>
       <c r="C17" s="159" t="n">
@@ -3129,17 +3129,17 @@
       </c>
       <c r="D17" s="158" t="inlineStr">
         <is>
-          <t>IDM</t>
+          <t>BR1</t>
         </is>
       </c>
       <c r="E17" s="158" t="inlineStr">
         <is>
-          <t>555</t>
+          <t>99955</t>
         </is>
       </c>
       <c r="F17" s="158" t="inlineStr">
         <is>
-          <t>MLD</t>
+          <t>LOC1</t>
         </is>
       </c>
       <c r="G17" s="158" t="n"/>
@@ -3202,7 +3202,7 @@
       </c>
       <c r="B18" s="158" t="inlineStr">
         <is>
-          <t>1000000.141000.CC</t>
+          <t>9100000.611000.A1</t>
         </is>
       </c>
       <c r="C18" s="159" t="n">
@@ -3210,17 +3210,17 @@
       </c>
       <c r="D18" s="158" t="inlineStr">
         <is>
-          <t>IDM</t>
+          <t>BR1</t>
         </is>
       </c>
       <c r="E18" s="158" t="inlineStr">
         <is>
-          <t>555</t>
+          <t>99955</t>
         </is>
       </c>
       <c r="F18" s="158" t="inlineStr">
         <is>
-          <t>MLD</t>
+          <t>LOC1</t>
         </is>
       </c>
       <c r="G18" s="158" t="n"/>
@@ -3241,7 +3241,7 @@
       </c>
       <c r="K18" s="158" t="inlineStr">
         <is>
-          <t>WHS A MLD</t>
+          <t>WHS A LOC1</t>
         </is>
       </c>
       <c r="L18" s="161" t="n">
@@ -3283,7 +3283,7 @@
       </c>
       <c r="B19" s="158" t="inlineStr">
         <is>
-          <t>1000000.141000.CC</t>
+          <t>9100000.611000.A1</t>
         </is>
       </c>
       <c r="C19" s="159" t="n">
@@ -3291,17 +3291,17 @@
       </c>
       <c r="D19" s="158" t="inlineStr">
         <is>
-          <t>IDM</t>
+          <t>BR1</t>
         </is>
       </c>
       <c r="E19" s="158" t="inlineStr">
         <is>
-          <t>555</t>
+          <t>99955</t>
         </is>
       </c>
       <c r="F19" s="158" t="inlineStr">
         <is>
-          <t>MLD</t>
+          <t>LOC1</t>
         </is>
       </c>
       <c r="G19" s="158" t="n"/>
@@ -3364,7 +3364,7 @@
       </c>
       <c r="B20" s="158" t="inlineStr">
         <is>
-          <t>1000000.141000.CC</t>
+          <t>9100000.611000.A1</t>
         </is>
       </c>
       <c r="C20" s="159" t="n">
@@ -3372,17 +3372,17 @@
       </c>
       <c r="D20" s="158" t="inlineStr">
         <is>
-          <t>IDM</t>
+          <t>BR1</t>
         </is>
       </c>
       <c r="E20" s="158" t="inlineStr">
         <is>
-          <t>555</t>
+          <t>99955</t>
         </is>
       </c>
       <c r="F20" s="158" t="inlineStr">
         <is>
-          <t>MLD</t>
+          <t>LOC1</t>
         </is>
       </c>
       <c r="G20" s="158" t="n"/>
@@ -3445,7 +3445,7 @@
       </c>
       <c r="B21" s="165" t="inlineStr">
         <is>
-          <t>1000000.141000.CC</t>
+          <t>9100000.611000.A1</t>
         </is>
       </c>
       <c r="C21" s="166" t="n">
@@ -3453,17 +3453,17 @@
       </c>
       <c r="D21" s="165" t="inlineStr">
         <is>
-          <t>IDM</t>
+          <t>BR1</t>
         </is>
       </c>
       <c r="E21" s="165" t="inlineStr">
         <is>
-          <t>555</t>
+          <t>99955</t>
         </is>
       </c>
       <c r="F21" s="165" t="inlineStr">
         <is>
-          <t>MLD</t>
+          <t>LOC1</t>
         </is>
       </c>
       <c r="G21" s="165" t="n"/>
@@ -3526,7 +3526,7 @@
       </c>
       <c r="B22" s="172" t="inlineStr">
         <is>
-          <t>1000000.141000.CC</t>
+          <t>9100000.611000.A1</t>
         </is>
       </c>
       <c r="C22" s="173" t="n">
@@ -3534,17 +3534,17 @@
       </c>
       <c r="D22" s="172" t="inlineStr">
         <is>
-          <t>IDM</t>
+          <t>BR1</t>
         </is>
       </c>
       <c r="E22" s="172" t="inlineStr">
         <is>
-          <t>555</t>
+          <t>99955</t>
         </is>
       </c>
       <c r="F22" s="172" t="inlineStr">
         <is>
-          <t>MLD</t>
+          <t>LOC1</t>
         </is>
       </c>
       <c r="G22" s="172" t="n"/>
@@ -3607,7 +3607,7 @@
       </c>
       <c r="B23" s="165" t="inlineStr">
         <is>
-          <t>1000000.141000.CC</t>
+          <t>9100000.611000.A1</t>
         </is>
       </c>
       <c r="C23" s="166" t="n">
@@ -3615,17 +3615,17 @@
       </c>
       <c r="D23" s="165" t="inlineStr">
         <is>
-          <t>IDM</t>
+          <t>BR1</t>
         </is>
       </c>
       <c r="E23" s="165" t="inlineStr">
         <is>
-          <t>555</t>
+          <t>99955</t>
         </is>
       </c>
       <c r="F23" s="165" t="inlineStr">
         <is>
-          <t>MLD</t>
+          <t>LOC1</t>
         </is>
       </c>
       <c r="G23" s="165" t="n"/>
@@ -3688,7 +3688,7 @@
       </c>
       <c r="B24" s="165" t="inlineStr">
         <is>
-          <t>1000000.141000.CC</t>
+          <t>9100000.611000.A1</t>
         </is>
       </c>
       <c r="C24" s="166" t="n">
@@ -3696,17 +3696,17 @@
       </c>
       <c r="D24" s="165" t="inlineStr">
         <is>
-          <t>IDM</t>
+          <t>BR1</t>
         </is>
       </c>
       <c r="E24" s="165" t="inlineStr">
         <is>
-          <t>555</t>
+          <t>99955</t>
         </is>
       </c>
       <c r="F24" s="165" t="inlineStr">
         <is>
-          <t>MLD</t>
+          <t>LOC1</t>
         </is>
       </c>
       <c r="G24" s="165" t="n"/>
@@ -3769,7 +3769,7 @@
       </c>
       <c r="B25" s="179" t="inlineStr">
         <is>
-          <t>1000000.141000.CC</t>
+          <t>9100000.611000.A1</t>
         </is>
       </c>
       <c r="C25" s="180" t="n">
@@ -3777,17 +3777,17 @@
       </c>
       <c r="D25" s="179" t="inlineStr">
         <is>
-          <t>IDM</t>
+          <t>BR1</t>
         </is>
       </c>
       <c r="E25" s="179" t="inlineStr">
         <is>
-          <t>555</t>
+          <t>99955</t>
         </is>
       </c>
       <c r="F25" s="179" t="inlineStr">
         <is>
-          <t>MLD</t>
+          <t>LOC1</t>
         </is>
       </c>
       <c r="G25" s="179" t="n"/>

</xml_diff>